<commit_message>
Add correlation trade-off analysis, dashboard Statistics tab, and Adult fidelity fixes.
Includes primary/supplementary Utility-Fidelity-Privacy figures for Cancer and Mushroom, utility-drop and representative trade-off modules, refreshed master/dashboard data, and Adult SDV Gower metrics from the live notebook.
</commit_message>
<xml_diff>
--- a/Generators/Experiment with utility data leak/utility results/13. Concrete Compressive Strength/TRTR_TSTR_results_merged.xlsx
+++ b/Generators/Experiment with utility data leak/utility results/13. Concrete Compressive Strength/TRTR_TSTR_results_merged.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Quality_Metrics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TRTR_Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="All_Comparisons" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CTGAN" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CopulaGAN" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TVAE" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GaussianCopula" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="WGAN_GP" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="CTABGAN" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TabDDPM" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ForestDiffusion" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality_Metrics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRTR_Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Comparisons" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CTGAN" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CopulaGAN" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TVAE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GaussianCopula" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WGAN_GP" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CTABGAN" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TabDDPM" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestDiffusion" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,13 +28,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -45,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,12 +56,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,22 +440,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Synthetic Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Quality Score</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Quality_Score</t>
         </is>
@@ -500,152 +512,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -1786,152 +1798,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -3072,152 +3084,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -4358,67 +4370,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)</t>
         </is>
@@ -4949,152 +4961,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -14075,27 +14087,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
@@ -14268,152 +14280,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -15554,152 +15566,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -16840,152 +16852,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -18126,152 +18138,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -19412,152 +19424,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>R2 Mean_TSTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>R2 Std_TSTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MSE Std_TSTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>RMSE Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RMSE Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MAE Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MAE Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>R2 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RMSE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MAE (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>R2_Drop</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MSE_Increase</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RMSE_Increase</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MAE_Increase</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>

</xml_diff>